<commit_message>
docs: add comprehensive demo Excel reports across inventory, finance, and registers
</commit_message>
<xml_diff>
--- a/docs/portfolio/assets/Kusum-ERP-demo-sales-register.xlsx
+++ b/docs/portfolio/assets/Kusum-ERP-demo-sales-register.xlsx
@@ -4,41 +4,50 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Data Export" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="All" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Gold" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Silver" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Data Export'!$A1:$J5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Data Export'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'All'!$A1:$M6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gold'!$A1:$M6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Gold'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Silver'!$A1:$M6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Silver'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Kusum Jewellers - Sales invoices</t>
-  </si>
-  <si>
-    <t>Portfolio sample register | 20-Sep-26 to 20-Sep-26</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Doc-no</t>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Gr-wt</t>
-  </si>
-  <si>
-    <t>Net-wt</t>
-  </si>
-  <si>
-    <t>Taxable-amt</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="21">
+  <si>
+    <t>Kusum Jewellers</t>
+  </si>
+  <si>
+    <t>ALL SALES REGISTER</t>
+  </si>
+  <si>
+    <t>Portfolio sample | 2026-09-20</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>DOC-NO</t>
+  </si>
+  <si>
+    <t>CUSTOMER</t>
+  </si>
+  <si>
+    <t>GR-WT</t>
+  </si>
+  <si>
+    <t>NET-WT</t>
+  </si>
+  <si>
+    <t>TAXABLE-AMT</t>
   </si>
   <si>
     <t>CGST</t>
@@ -47,10 +56,19 @@
     <t>SGST</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Payment</t>
+    <t>IGST</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>URD</t>
+  </si>
+  <si>
+    <t>DISCOUNT</t>
+  </si>
+  <si>
+    <t>NET-AMT</t>
   </si>
   <si>
     <r>
@@ -61,7 +79,13 @@
     <t>Parikshit Abuj</t>
   </si>
   <si>
-    <t>Cash + UPI</t>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>GOLD SALES REGISTER</t>
+  </si>
+  <si>
+    <t>SILVER SALES REGISTER</t>
   </si>
 </sst>
 </file>
@@ -69,10 +93,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000;[Red]-0.000"/>
-    <numFmt numFmtId="165" formatCode="[$₹-en-IN]#,##0.00;[Red]-[$₹-en-IN]#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000;[Red]-#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -82,43 +106,41 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <sz val="16"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF756F69"/>
-      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF271A05"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF30251D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD5A044"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -126,62 +148,47 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD2B77F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD2B77F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD2B77F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD2B77F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFE8E1D8"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFE8E1D8"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE8E1D8"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE8E1D8"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -526,20 +533,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="6" max="13" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,8 +556,11 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -566,82 +573,545 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="G4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="H4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="I4" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
         <v>46285.5</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="B5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="9">
         <v>25.2</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>22.85</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="10">
         <v>42067.2</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>631.01</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <v>631.01</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="10">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10">
         <v>43329.22</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>14</v>
+      <c r="K5" s="10">
+        <v>0</v>
+      </c>
+      <c r="L5" s="10">
+        <v>0</v>
+      </c>
+      <c r="M5" s="10">
+        <v>43329.22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="12">
+        <f>SUM(D5:D5)</f>
+        <v>25.2</v>
+      </c>
+      <c r="E6" s="12">
+        <f>SUM(E5:E5)</f>
+        <v>22.85</v>
+      </c>
+      <c r="F6" s="13">
+        <f>SUM(F5:F5)</f>
+        <v>42067.2</v>
+      </c>
+      <c r="G6" s="13">
+        <f>SUM(G5:G5)</f>
+        <v>631.01</v>
+      </c>
+      <c r="H6" s="13">
+        <f>SUM(H5:H5)</f>
+        <v>631.01</v>
+      </c>
+      <c r="I6" s="13">
+        <f>SUM(I5:I5)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="13">
+        <f>SUM(J5:J5)</f>
+        <v>43329.22</v>
+      </c>
+      <c r="K6" s="13">
+        <f>SUM(K5:K5)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>SUM(L5:L5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="13">
+        <f>SUM(M5:M5)</f>
+        <v>43329.22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J5"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
-  <headerFooter>
-    <oddFooter>&amp;LKusum Jewellers&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</oddFooter>
-    <evenFooter>&amp;LKusum Jewellers&amp;CConfidential business register&amp;RPage &amp;P of &amp;N</evenFooter>
-  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="5" width="13" customWidth="1"/>
+    <col min="6" max="13" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>46285.5</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="9">
+        <v>5.2</v>
+      </c>
+      <c r="E5" s="9">
+        <v>4.85</v>
+      </c>
+      <c r="F5" s="10">
+        <v>39925.2</v>
+      </c>
+      <c r="G5" s="10">
+        <v>598.88</v>
+      </c>
+      <c r="H5" s="10">
+        <v>598.88</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10">
+        <v>41122.96</v>
+      </c>
+      <c r="K5" s="10">
+        <v>0</v>
+      </c>
+      <c r="L5" s="10">
+        <v>0</v>
+      </c>
+      <c r="M5" s="10">
+        <v>41122.96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="12">
+        <f>SUM(D5:D5)</f>
+        <v>5.2</v>
+      </c>
+      <c r="E6" s="12">
+        <f>SUM(E5:E5)</f>
+        <v>4.85</v>
+      </c>
+      <c r="F6" s="13">
+        <f>SUM(F5:F5)</f>
+        <v>39925.2</v>
+      </c>
+      <c r="G6" s="13">
+        <f>SUM(G5:G5)</f>
+        <v>598.88</v>
+      </c>
+      <c r="H6" s="13">
+        <f>SUM(H5:H5)</f>
+        <v>598.88</v>
+      </c>
+      <c r="J6" s="13">
+        <f>SUM(J5:J5)</f>
+        <v>41122.96</v>
+      </c>
+      <c r="M6" s="13">
+        <f>SUM(M5:M5)</f>
+        <v>41122.96</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="5" width="13" customWidth="1"/>
+    <col min="6" max="13" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>46285.5</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="9">
+        <v>20</v>
+      </c>
+      <c r="E5" s="9">
+        <v>18</v>
+      </c>
+      <c r="F5" s="10">
+        <v>2142</v>
+      </c>
+      <c r="G5" s="10">
+        <v>32.13</v>
+      </c>
+      <c r="H5" s="10">
+        <v>32.13</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0</v>
+      </c>
+      <c r="J5" s="10">
+        <v>2206.26</v>
+      </c>
+      <c r="K5" s="10">
+        <v>0</v>
+      </c>
+      <c r="L5" s="10">
+        <v>0</v>
+      </c>
+      <c r="M5" s="10">
+        <v>2206.26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="12">
+        <f>SUM(D5:D5)</f>
+        <v>20</v>
+      </c>
+      <c r="E6" s="12">
+        <f>SUM(E5:E5)</f>
+        <v>18</v>
+      </c>
+      <c r="F6" s="13">
+        <f>SUM(F5:F5)</f>
+        <v>2142</v>
+      </c>
+      <c r="G6" s="13">
+        <f>SUM(G5:G5)</f>
+        <v>32.13</v>
+      </c>
+      <c r="H6" s="13">
+        <f>SUM(H5:H5)</f>
+        <v>32.13</v>
+      </c>
+      <c r="J6" s="13">
+        <f>SUM(J5:J5)</f>
+        <v>2206.26</v>
+      </c>
+      <c r="M6" s="13">
+        <f>SUM(M5:M5)</f>
+        <v>2206.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>